<commit_message>
v1.1.0: tz-aware date conversion (default America/Los_Angeles), --tz flag, interactive PT warning, src/diag_pr.py helper for debugging missed PRs
</commit_message>
<xml_diff>
--- a/Monthly Report Data.xlsx
+++ b/Monthly Report Data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/amandalapu/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/amandalapu/Personal/pr-sla-report/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18127F4F-87BA-4F40-A149-1FC9D2DDB9C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FD81408-EA43-C246-9840-E577D817244D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17740" activeTab="2" xr2:uid="{D5970AE5-8A85-8C48-A57F-72444ABEF9C2}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17740" activeTab="1" xr2:uid="{D5970AE5-8A85-8C48-A57F-72444ABEF9C2}"/>
   </bookViews>
   <sheets>
     <sheet name="Repos" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="58">
   <si>
     <t>ADO Repo</t>
   </si>
@@ -354,6 +354,12 @@
       </rPr>
       <t>​</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">v-aprasadpuj@microsoft.com </t>
+  </si>
+  <si>
+    <t>Ahobila Pavana Lakshmi N R Prasad Pujari</t>
   </si>
 </sst>
 </file>
@@ -804,7 +810,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12EB12EC-6E9C-E048-9598-800C4D30E699}">
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.1640625" bestFit="1" customWidth="1"/>
@@ -821,114 +827,123 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>57</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>6</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
         <v>27</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B14" s="1" t="s">
         <v>28</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" xr:uid="{AF773801-B675-C445-82BB-8555D1AAA1C9}"/>
-    <hyperlink ref="B3" r:id="rId2" xr:uid="{A11B9943-4D09-0745-AE04-B9003D04D273}"/>
-    <hyperlink ref="B4" r:id="rId3" xr:uid="{E51B2865-0006-D04B-8DB9-10241EBCACA2}"/>
-    <hyperlink ref="B5" r:id="rId4" xr:uid="{CBDABB10-232B-624C-AB6D-20DBD15367DE}"/>
-    <hyperlink ref="B6" r:id="rId5" xr:uid="{E2FD91EC-9B71-E649-895C-575D7EEA1ED1}"/>
-    <hyperlink ref="B7" r:id="rId6" xr:uid="{99A6903D-29B8-4A41-B4A8-11DE627A6C25}"/>
-    <hyperlink ref="B8" r:id="rId7" xr:uid="{C7906ABF-CD00-3D46-A007-334AF4A84251}"/>
-    <hyperlink ref="B9" r:id="rId8" xr:uid="{B236ADF2-F099-664A-94E7-2EE828337C7E}"/>
-    <hyperlink ref="B10" r:id="rId9" xr:uid="{DB347399-CC71-784C-90F3-9ADAFCE0EAD3}"/>
-    <hyperlink ref="B11" r:id="rId10" xr:uid="{2750F001-F127-6042-B5E6-F59F679BAE6F}"/>
-    <hyperlink ref="B12" r:id="rId11" xr:uid="{17339EBE-08A5-C74E-9275-E6B63325D8CC}"/>
-    <hyperlink ref="B13" r:id="rId12" xr:uid="{E2A45B26-16B2-EC44-8EA4-6A901463DAEA}"/>
+    <hyperlink ref="B3" r:id="rId1" xr:uid="{AF773801-B675-C445-82BB-8555D1AAA1C9}"/>
+    <hyperlink ref="B4" r:id="rId2" xr:uid="{A11B9943-4D09-0745-AE04-B9003D04D273}"/>
+    <hyperlink ref="B5" r:id="rId3" xr:uid="{E51B2865-0006-D04B-8DB9-10241EBCACA2}"/>
+    <hyperlink ref="B6" r:id="rId4" xr:uid="{CBDABB10-232B-624C-AB6D-20DBD15367DE}"/>
+    <hyperlink ref="B7" r:id="rId5" xr:uid="{E2FD91EC-9B71-E649-895C-575D7EEA1ED1}"/>
+    <hyperlink ref="B8" r:id="rId6" xr:uid="{99A6903D-29B8-4A41-B4A8-11DE627A6C25}"/>
+    <hyperlink ref="B9" r:id="rId7" xr:uid="{C7906ABF-CD00-3D46-A007-334AF4A84251}"/>
+    <hyperlink ref="B10" r:id="rId8" xr:uid="{B236ADF2-F099-664A-94E7-2EE828337C7E}"/>
+    <hyperlink ref="B11" r:id="rId9" xr:uid="{DB347399-CC71-784C-90F3-9ADAFCE0EAD3}"/>
+    <hyperlink ref="B12" r:id="rId10" xr:uid="{2750F001-F127-6042-B5E6-F59F679BAE6F}"/>
+    <hyperlink ref="B13" r:id="rId11" xr:uid="{17339EBE-08A5-C74E-9275-E6B63325D8CC}"/>
+    <hyperlink ref="B14" r:id="rId12" xr:uid="{E2A45B26-16B2-EC44-8EA4-6A901463DAEA}"/>
+    <hyperlink ref="B2" r:id="rId13" xr:uid="{F8DBEB9C-2795-D74F-85D6-7BA3E31F8C76}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1137,11 +1152,36 @@
     </row>
   </sheetData>
   <mergeCells count="42">
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="D13:D14"/>
-    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="E3:E4"/>
+    <mergeCell ref="F3:F4"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="E9:E10"/>
     <mergeCell ref="F13:F14"/>
     <mergeCell ref="A11:A12"/>
     <mergeCell ref="B11:B12"/>
@@ -1149,36 +1189,11 @@
     <mergeCell ref="D11:D12"/>
     <mergeCell ref="E11:E12"/>
     <mergeCell ref="F11:F12"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="D7:D8"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="F7:F8"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="E3:E4"/>
-    <mergeCell ref="F3:F4"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="E13:E14"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A3" r:id="rId1" display="https://dev.azure.com/MicrosoftIT/OneITVSO/_workitems/edit/15837038/" xr:uid="{D691395E-6EE0-2140-ADF5-F09C0471ED12}"/>

</xml_diff>

<commit_message>
v1.3.0: bearer-token auth via az CLI (no PAT in dotfiles); auto-resolver tries ADO_PAT then az then errors; interactive runner offers az before PAT
</commit_message>
<xml_diff>
--- a/Monthly Report Data.xlsx
+++ b/Monthly Report Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/amandalapu/Personal/pr-sla-report/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FD81408-EA43-C246-9840-E577D817244D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9BEDDA1-9027-1D4C-9090-8B2B1D8275AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17740" activeTab="1" xr2:uid="{D5970AE5-8A85-8C48-A57F-72444ABEF9C2}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="60">
   <si>
     <t>ADO Repo</t>
   </si>
@@ -360,6 +360,12 @@
   </si>
   <si>
     <t>Ahobila Pavana Lakshmi N R Prasad Pujari</t>
+  </si>
+  <si>
+    <t>Brajesh Chandra</t>
+  </si>
+  <si>
+    <t>v-brchandra@microsoft.com</t>
   </si>
 </sst>
 </file>
@@ -439,10 +445,10 @@
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -810,7 +816,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12EB12EC-6E9C-E048-9598-800C4D30E699}">
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.1640625" bestFit="1" customWidth="1"/>
@@ -851,81 +857,89 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>58</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>10</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
+        <v>25</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B15" s="1" t="s">
         <v>28</v>
       </c>
     </row>
@@ -933,17 +947,18 @@
   <hyperlinks>
     <hyperlink ref="B3" r:id="rId1" xr:uid="{AF773801-B675-C445-82BB-8555D1AAA1C9}"/>
     <hyperlink ref="B4" r:id="rId2" xr:uid="{A11B9943-4D09-0745-AE04-B9003D04D273}"/>
-    <hyperlink ref="B5" r:id="rId3" xr:uid="{E51B2865-0006-D04B-8DB9-10241EBCACA2}"/>
-    <hyperlink ref="B6" r:id="rId4" xr:uid="{CBDABB10-232B-624C-AB6D-20DBD15367DE}"/>
-    <hyperlink ref="B7" r:id="rId5" xr:uid="{E2FD91EC-9B71-E649-895C-575D7EEA1ED1}"/>
-    <hyperlink ref="B8" r:id="rId6" xr:uid="{99A6903D-29B8-4A41-B4A8-11DE627A6C25}"/>
-    <hyperlink ref="B9" r:id="rId7" xr:uid="{C7906ABF-CD00-3D46-A007-334AF4A84251}"/>
-    <hyperlink ref="B10" r:id="rId8" xr:uid="{B236ADF2-F099-664A-94E7-2EE828337C7E}"/>
-    <hyperlink ref="B11" r:id="rId9" xr:uid="{DB347399-CC71-784C-90F3-9ADAFCE0EAD3}"/>
-    <hyperlink ref="B12" r:id="rId10" xr:uid="{2750F001-F127-6042-B5E6-F59F679BAE6F}"/>
-    <hyperlink ref="B13" r:id="rId11" xr:uid="{17339EBE-08A5-C74E-9275-E6B63325D8CC}"/>
-    <hyperlink ref="B14" r:id="rId12" xr:uid="{E2A45B26-16B2-EC44-8EA4-6A901463DAEA}"/>
+    <hyperlink ref="B6" r:id="rId3" xr:uid="{E51B2865-0006-D04B-8DB9-10241EBCACA2}"/>
+    <hyperlink ref="B7" r:id="rId4" xr:uid="{CBDABB10-232B-624C-AB6D-20DBD15367DE}"/>
+    <hyperlink ref="B8" r:id="rId5" xr:uid="{E2FD91EC-9B71-E649-895C-575D7EEA1ED1}"/>
+    <hyperlink ref="B9" r:id="rId6" xr:uid="{99A6903D-29B8-4A41-B4A8-11DE627A6C25}"/>
+    <hyperlink ref="B10" r:id="rId7" xr:uid="{C7906ABF-CD00-3D46-A007-334AF4A84251}"/>
+    <hyperlink ref="B11" r:id="rId8" xr:uid="{B236ADF2-F099-664A-94E7-2EE828337C7E}"/>
+    <hyperlink ref="B12" r:id="rId9" xr:uid="{DB347399-CC71-784C-90F3-9ADAFCE0EAD3}"/>
+    <hyperlink ref="B13" r:id="rId10" xr:uid="{2750F001-F127-6042-B5E6-F59F679BAE6F}"/>
+    <hyperlink ref="B14" r:id="rId11" xr:uid="{17339EBE-08A5-C74E-9275-E6B63325D8CC}"/>
+    <hyperlink ref="B15" r:id="rId12" xr:uid="{E2A45B26-16B2-EC44-8EA4-6A901463DAEA}"/>
     <hyperlink ref="B2" r:id="rId13" xr:uid="{F8DBEB9C-2795-D74F-85D6-7BA3E31F8C76}"/>
+    <hyperlink ref="B5" r:id="rId14" xr:uid="{4077F0E4-5A87-E242-B96A-7E717819C7DA}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -955,35 +970,35 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="2" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" s="5"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="4" t="s">
         <v>29</v>
       </c>
       <c r="B3" s="3" t="s">
@@ -1003,7 +1018,7 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4" s="2"/>
+      <c r="A4" s="4"/>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
@@ -1011,7 +1026,7 @@
       <c r="F4" s="3"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="5" t="s">
         <v>35</v>
       </c>
       <c r="B5" s="3" t="s">
@@ -1031,7 +1046,7 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A6" s="4"/>
+      <c r="A6" s="5"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
@@ -1039,7 +1054,7 @@
       <c r="F6" s="3"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="5" t="s">
         <v>39</v>
       </c>
       <c r="B7" s="3" t="s">
@@ -1059,7 +1074,7 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A8" s="4"/>
+      <c r="A8" s="5"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
       <c r="D8" s="3"/>
@@ -1067,7 +1082,7 @@
       <c r="F8" s="3"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="4" t="s">
         <v>42</v>
       </c>
       <c r="B9" s="3" t="s">
@@ -1087,7 +1102,7 @@
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A10" s="2"/>
+      <c r="A10" s="4"/>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
       <c r="D10" s="3"/>
@@ -1095,7 +1110,7 @@
       <c r="F10" s="3"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="4" t="s">
         <v>45</v>
       </c>
       <c r="B11" s="3" t="s">
@@ -1115,7 +1130,7 @@
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A12" s="2"/>
+      <c r="A12" s="4"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
@@ -1123,7 +1138,7 @@
       <c r="F12" s="3"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="4" t="s">
         <v>47</v>
       </c>
       <c r="B13" s="3" t="s">
@@ -1143,7 +1158,7 @@
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A14" s="2"/>
+      <c r="A14" s="4"/>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
@@ -1152,12 +1167,30 @@
     </row>
   </sheetData>
   <mergeCells count="42">
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F13:F14"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="E9:E10"/>
     <mergeCell ref="F5:F6"/>
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="B3:B4"/>
@@ -1170,30 +1203,12 @@
     <mergeCell ref="C5:C6"/>
     <mergeCell ref="D5:D6"/>
     <mergeCell ref="E5:E6"/>
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="D7:D8"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="F7:F8"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="F13:F14"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="F11:F12"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="D13:D14"/>
-    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:E2"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A3" r:id="rId1" display="https://dev.azure.com/MicrosoftIT/OneITVSO/_workitems/edit/15837038/" xr:uid="{D691395E-6EE0-2140-ADF5-F09C0471ED12}"/>

</xml_diff>

<commit_message>
Add opt-in filtering for PRs exceeding two business days
Include shared holiday setup, filtered report naming, regression tests, documentation, and updated report workbook.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Monthly Report Data.xlsx
+++ b/Monthly Report Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/amandalapu/Personal/pr-sla-report/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9BEDDA1-9027-1D4C-9090-8B2B1D8275AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAE731D1-A8C6-B64E-AD11-26394D722E69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17740" activeTab="1" xr2:uid="{D5970AE5-8A85-8C48-A57F-72444ABEF9C2}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17500" activeTab="1" xr2:uid="{D5970AE5-8A85-8C48-A57F-72444ABEF9C2}"/>
   </bookViews>
   <sheets>
     <sheet name="Repos" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="62">
   <si>
     <t>ADO Repo</t>
   </si>
@@ -58,34 +58,16 @@
     <t>V-id</t>
   </si>
   <si>
-    <t xml:space="preserve">Akshay Lagad </t>
-  </si>
-  <si>
-    <t>v-aklagad@microsoft.com</t>
-  </si>
-  <si>
     <t>Avinash MANDALAPU</t>
   </si>
   <si>
     <t>v-avinashman@microsoft.com</t>
   </si>
   <si>
-    <t>JONNA ANAND</t>
-  </si>
-  <si>
-    <t>v-jonnaanand@microsoft.com</t>
-  </si>
-  <si>
     <t>Khushi Mandle</t>
   </si>
   <si>
     <t>v-kmandle@microsoft.com</t>
-  </si>
-  <si>
-    <t>Kolanu Jagadeesh Sai</t>
-  </si>
-  <si>
-    <t>v-kolasai@microsoft.com</t>
   </si>
   <si>
     <t>Manimaran Annamalai</t>
@@ -356,16 +338,40 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">v-aprasadpuj@microsoft.com </t>
-  </si>
-  <si>
-    <t>Ahobila Pavana Lakshmi N R Prasad Pujari</t>
-  </si>
-  <si>
     <t>Brajesh Chandra</t>
   </si>
   <si>
     <t>v-brchandra@microsoft.com</t>
+  </si>
+  <si>
+    <t>v-anjuc@microsoft.com</t>
+  </si>
+  <si>
+    <t>Anju Chaturvedi</t>
+  </si>
+  <si>
+    <t>Dilpreet Singh Rajpal</t>
+  </si>
+  <si>
+    <t>v-drajpal@microsoft.com</t>
+  </si>
+  <si>
+    <t>Mohan Sundar S</t>
+  </si>
+  <si>
+    <t>v-mohansus@microsoft.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Souvik Chakraborty </t>
+  </si>
+  <si>
+    <t>v-chsouvik@microsoft.com</t>
+  </si>
+  <si>
+    <t>v-yashshr@microsoft.com</t>
+  </si>
+  <si>
+    <t>Yash Shrivastava</t>
   </si>
 </sst>
 </file>
@@ -816,7 +822,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12EB12EC-6E9C-E048-9598-800C4D30E699}">
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.1640625" bestFit="1" customWidth="1"/>
@@ -833,18 +839,18 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>57</v>
+        <v>5</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>56</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>6</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -857,108 +863,117 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>58</v>
+        <v>9</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>59</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>21</v>
+        <v>53</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>22</v>
+        <v>52</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>54</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>24</v>
+        <v>55</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>25</v>
+        <v>56</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>26</v>
+        <v>57</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>27</v>
+        <v>58</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>28</v>
+        <v>59</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>61</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>60</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B3" r:id="rId1" xr:uid="{AF773801-B675-C445-82BB-8555D1AAA1C9}"/>
-    <hyperlink ref="B4" r:id="rId2" xr:uid="{A11B9943-4D09-0745-AE04-B9003D04D273}"/>
-    <hyperlink ref="B6" r:id="rId3" xr:uid="{E51B2865-0006-D04B-8DB9-10241EBCACA2}"/>
-    <hyperlink ref="B7" r:id="rId4" xr:uid="{CBDABB10-232B-624C-AB6D-20DBD15367DE}"/>
-    <hyperlink ref="B8" r:id="rId5" xr:uid="{E2FD91EC-9B71-E649-895C-575D7EEA1ED1}"/>
-    <hyperlink ref="B9" r:id="rId6" xr:uid="{99A6903D-29B8-4A41-B4A8-11DE627A6C25}"/>
-    <hyperlink ref="B10" r:id="rId7" xr:uid="{C7906ABF-CD00-3D46-A007-334AF4A84251}"/>
-    <hyperlink ref="B11" r:id="rId8" xr:uid="{B236ADF2-F099-664A-94E7-2EE828337C7E}"/>
-    <hyperlink ref="B12" r:id="rId9" xr:uid="{DB347399-CC71-784C-90F3-9ADAFCE0EAD3}"/>
-    <hyperlink ref="B13" r:id="rId10" xr:uid="{2750F001-F127-6042-B5E6-F59F679BAE6F}"/>
-    <hyperlink ref="B14" r:id="rId11" xr:uid="{17339EBE-08A5-C74E-9275-E6B63325D8CC}"/>
-    <hyperlink ref="B15" r:id="rId12" xr:uid="{E2A45B26-16B2-EC44-8EA4-6A901463DAEA}"/>
-    <hyperlink ref="B2" r:id="rId13" xr:uid="{F8DBEB9C-2795-D74F-85D6-7BA3E31F8C76}"/>
-    <hyperlink ref="B5" r:id="rId14" xr:uid="{4077F0E4-5A87-E242-B96A-7E717819C7DA}"/>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{A11B9943-4D09-0745-AE04-B9003D04D273}"/>
+    <hyperlink ref="B4" r:id="rId2" xr:uid="{CBDABB10-232B-624C-AB6D-20DBD15367DE}"/>
+    <hyperlink ref="B5" r:id="rId3" xr:uid="{99A6903D-29B8-4A41-B4A8-11DE627A6C25}"/>
+    <hyperlink ref="B6" r:id="rId4" xr:uid="{C7906ABF-CD00-3D46-A007-334AF4A84251}"/>
+    <hyperlink ref="B7" r:id="rId5" xr:uid="{B236ADF2-F099-664A-94E7-2EE828337C7E}"/>
+    <hyperlink ref="B8" r:id="rId6" xr:uid="{DB347399-CC71-784C-90F3-9ADAFCE0EAD3}"/>
+    <hyperlink ref="B9" r:id="rId7" xr:uid="{2750F001-F127-6042-B5E6-F59F679BAE6F}"/>
+    <hyperlink ref="B10" r:id="rId8" xr:uid="{17339EBE-08A5-C74E-9275-E6B63325D8CC}"/>
+    <hyperlink ref="B11" r:id="rId9" xr:uid="{E2A45B26-16B2-EC44-8EA4-6A901463DAEA}"/>
+    <hyperlink ref="B3" r:id="rId10" xr:uid="{4077F0E4-5A87-E242-B96A-7E717819C7DA}"/>
+    <hyperlink ref="B12" r:id="rId11" xr:uid="{425DD7DF-0707-4B49-BB76-9D96B4FE4F6B}"/>
+    <hyperlink ref="B13" r:id="rId12" xr:uid="{5DED3772-4569-E841-A4E8-0C64A67D972C}"/>
+    <hyperlink ref="B14" r:id="rId13" xr:uid="{B4D30D76-25BA-2143-B037-7797853AA8FB}"/>
+    <hyperlink ref="B15" r:id="rId14" xr:uid="{D5ECE8DB-A5DA-164D-9C4E-85A68E166C4E}"/>
+    <hyperlink ref="B16" r:id="rId15" xr:uid="{AACC7591-DAA7-8441-8431-7087E08C7AFE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -971,22 +986,22 @@
   <sheetData>
     <row r="1" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
@@ -999,22 +1014,22 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -1027,22 +1042,22 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -1055,22 +1070,22 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
@@ -1083,22 +1098,22 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -1111,22 +1126,22 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
@@ -1139,22 +1154,22 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">

</xml_diff>